<commit_message>
auto update (Home Full Ver)
</commit_message>
<xml_diff>
--- a/weekly_performance.xlsx
+++ b/weekly_performance.xlsx
@@ -876,22 +876,22 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E10" t="n">
-        <v>10.7</v>
+        <v>13.8</v>
       </c>
       <c r="F10" t="n">
-        <v>0.42</v>
+        <v>0.31</v>
       </c>
       <c r="G10" t="n">
-        <v>0.66</v>
+        <v>1.07</v>
       </c>
       <c r="H10" t="n">
         <v>0.65</v>
       </c>
       <c r="I10" t="n">
-        <v>0.9</v>
+        <v>2.29</v>
       </c>
       <c r="J10" t="n">
         <v>2.25</v>
@@ -899,7 +899,7 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
-        <v>-264819</v>
+        <v>-264788</v>
       </c>
     </row>
     <row r="11">
@@ -919,16 +919,16 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>34.8</v>
+        <v>35.1</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>2.05</v>
+        <v>2.03</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>4.28</v>
+        <v>4.25</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>2.26</v>
@@ -942,7 +942,7 @@
       <c r="K11" s="2" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="n">
-        <v>138598</v>
+        <v>138630</v>
       </c>
     </row>
     <row r="13">
@@ -1603,26 +1603,26 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E32" t="n">
         <v>100</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="n">
-        <v>0.55</v>
+        <v>1.13</v>
       </c>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="n">
-        <v>0.9</v>
+        <v>2.29</v>
       </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
-        <v>6</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33">
@@ -1642,34 +1642,34 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>30</v>
+        <v>36.4</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0.32</v>
+        <v>1.44</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>0.85</v>
+        <v>1.21</v>
       </c>
       <c r="H33" s="2" t="n">
         <v>1.02</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>1.46</v>
+        <v>2.29</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>3.41</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>8.33</v>
+        <v>10.75</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>4.29</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>-40</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
auto update (Company KR Ver)
</commit_message>
<xml_diff>
--- a/weekly_performance.xlsx
+++ b/weekly_performance.xlsx
@@ -878,19 +878,19 @@
         <v>3.19</v>
       </c>
       <c r="N7" t="n">
-        <v>31602</v>
+        <v>31601</v>
       </c>
       <c r="O7" t="n">
-        <v>11.33</v>
+        <v>11.32</v>
       </c>
       <c r="P7" t="n">
-        <v>379229</v>
+        <v>379217</v>
       </c>
       <c r="Q7" t="n">
         <v>2168</v>
       </c>
       <c r="R7" t="n">
-        <v>381397</v>
+        <v>381386</v>
       </c>
     </row>
     <row r="8">
@@ -936,19 +936,19 @@
         <v>1.549</v>
       </c>
       <c r="N8" t="n">
-        <v>3280</v>
+        <v>3278</v>
       </c>
       <c r="O8" t="n">
         <v>1.7</v>
       </c>
       <c r="P8" t="n">
-        <v>65607</v>
+        <v>65570</v>
       </c>
       <c r="Q8" t="n">
-        <v>7203</v>
+        <v>7207</v>
       </c>
       <c r="R8" t="n">
-        <v>72811</v>
+        <v>72777</v>
       </c>
     </row>
     <row r="9">
@@ -1000,13 +1000,13 @@
         <v>0.9</v>
       </c>
       <c r="P9" t="n">
-        <v>-17462</v>
+        <v>-17465</v>
       </c>
       <c r="Q9" t="n">
-        <v>8322</v>
+        <v>8324</v>
       </c>
       <c r="R9" t="n">
-        <v>-9140</v>
+        <v>-9141</v>
       </c>
     </row>
     <row r="10">
@@ -1052,19 +1052,19 @@
         <v>-0.448</v>
       </c>
       <c r="N10" t="n">
-        <v>-7903</v>
+        <v>-7902</v>
       </c>
       <c r="O10" t="n">
         <v>0.21</v>
       </c>
       <c r="P10" t="n">
-        <v>-229180</v>
+        <v>-229146</v>
       </c>
       <c r="Q10" t="n">
-        <v>17298</v>
+        <v>17301</v>
       </c>
       <c r="R10" t="n">
-        <v>-211882</v>
+        <v>-211845</v>
       </c>
     </row>
     <row r="11">
@@ -1116,13 +1116,13 @@
         <v>1.05</v>
       </c>
       <c r="P11" s="2" t="n">
-        <v>73719</v>
+        <v>73701</v>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>53141</v>
+        <v>53151</v>
       </c>
       <c r="R11" s="2" t="n">
-        <v>126860</v>
+        <v>126852</v>
       </c>
     </row>
     <row r="13">
@@ -1844,19 +1844,19 @@
         <v>-2.607</v>
       </c>
       <c r="N29" t="n">
-        <v>-8033</v>
+        <v>-8039</v>
       </c>
       <c r="O29" t="n">
         <v>0</v>
       </c>
       <c r="P29" t="n">
-        <v>-16066</v>
+        <v>-16078</v>
       </c>
       <c r="Q29" t="n">
         <v>514</v>
       </c>
       <c r="R29" t="n">
-        <v>-15552</v>
+        <v>-15563</v>
       </c>
     </row>
     <row r="30">
@@ -1906,19 +1906,19 @@
         <v>-0.217</v>
       </c>
       <c r="N30" t="n">
-        <v>-13310</v>
+        <v>-13319</v>
       </c>
       <c r="O30" t="n">
         <v>0.02</v>
       </c>
       <c r="P30" t="n">
-        <v>-53239</v>
+        <v>-53277</v>
       </c>
       <c r="Q30" t="n">
-        <v>5930</v>
+        <v>5934</v>
       </c>
       <c r="R30" t="n">
-        <v>-47309</v>
+        <v>-47343</v>
       </c>
     </row>
     <row r="31">
@@ -1962,19 +1962,19 @@
         <v>-0.136</v>
       </c>
       <c r="N31" t="n">
-        <v>-2395</v>
+        <v>-2397</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
       </c>
       <c r="P31" t="n">
-        <v>-4791</v>
+        <v>-4794</v>
       </c>
       <c r="Q31" t="n">
-        <v>2932</v>
+        <v>2934</v>
       </c>
       <c r="R31" t="n">
-        <v>-1859</v>
+        <v>-1860</v>
       </c>
     </row>
     <row r="32">
@@ -2016,17 +2016,17 @@
         <v>1.042</v>
       </c>
       <c r="N32" t="n">
-        <v>16226</v>
+        <v>16237</v>
       </c>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="n">
-        <v>48677</v>
+        <v>48711</v>
       </c>
       <c r="Q32" t="n">
-        <v>4266</v>
+        <v>4269</v>
       </c>
       <c r="R32" t="n">
-        <v>52943</v>
+        <v>52980</v>
       </c>
     </row>
     <row r="33">
@@ -2076,19 +2076,19 @@
         <v>-0.293</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-2311</v>
+        <v>-2312</v>
       </c>
       <c r="O33" s="2" t="n">
         <v>0.66</v>
       </c>
       <c r="P33" s="2" t="n">
-        <v>-25419</v>
+        <v>-25437</v>
       </c>
       <c r="Q33" s="2" t="n">
-        <v>13642</v>
+        <v>13651</v>
       </c>
       <c r="R33" s="2" t="n">
-        <v>-11778</v>
+        <v>-11786</v>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
report sync - 2026-08-16  9:41:45.73
</commit_message>
<xml_diff>
--- a/weekly_performance.xlsx
+++ b/weekly_performance.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R106"/>
+  <dimension ref="A1:S118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -455,6 +455,7 @@
     <col width="18" customWidth="1" min="16" max="16"/>
     <col width="15" customWidth="1" min="17" max="17"/>
     <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -548,6 +549,11 @@
           <t>실현손익합(원,gross)</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>환율(USDKRW)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -602,6 +608,9 @@
       <c r="R2" t="n">
         <v>-175500</v>
       </c>
+      <c r="S2" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -660,6 +669,9 @@
       <c r="R3" t="n">
         <v>229860</v>
       </c>
+      <c r="S3" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -718,6 +730,9 @@
       <c r="R4" t="n">
         <v>-219740</v>
       </c>
+      <c r="S4" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -776,6 +791,9 @@
       <c r="R5" t="n">
         <v>36101</v>
       </c>
+      <c r="S5" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -834,6 +852,9 @@
       <c r="R6" t="n">
         <v>26414</v>
       </c>
+      <c r="S6" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -892,6 +913,9 @@
       <c r="R7" t="n">
         <v>381441</v>
       </c>
+      <c r="S7" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -950,6 +974,9 @@
       <c r="R8" t="n">
         <v>72944</v>
       </c>
+      <c r="S8" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1008,6 +1035,9 @@
       <c r="R9" t="n">
         <v>-5715</v>
       </c>
+      <c r="S9" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1066,6 +1096,9 @@
       <c r="R10" t="n">
         <v>-172206</v>
       </c>
+      <c r="S10" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1090,7 +1123,7 @@
         <v>28.6</v>
       </c>
       <c r="F11" t="n">
-        <v>1.7</v>
+        <v>1.71</v>
       </c>
       <c r="G11" t="n">
         <v>8.56</v>
@@ -1110,19 +1143,22 @@
         <v>-0.327</v>
       </c>
       <c r="N11" t="n">
-        <v>-7689</v>
+        <v>-7621</v>
       </c>
       <c r="O11" t="n">
         <v>0.68</v>
       </c>
       <c r="P11" t="n">
-        <v>-53824</v>
+        <v>-53347</v>
       </c>
       <c r="Q11" t="n">
-        <v>15642</v>
+        <v>15600</v>
       </c>
       <c r="R11" t="n">
-        <v>-38182</v>
+        <v>-37747</v>
+      </c>
+      <c r="S11" t="n">
+        <v>1411</v>
       </c>
     </row>
     <row r="12">
@@ -1168,20 +1204,21 @@
         <v>-0.005</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="O12" s="2" t="n">
         <v>1.04</v>
       </c>
       <c r="P12" s="2" t="n">
-        <v>70396</v>
+        <v>70873</v>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>65020</v>
+        <v>64978</v>
       </c>
       <c r="R12" s="2" t="n">
-        <v>135416</v>
-      </c>
+        <v>135851</v>
+      </c>
+      <c r="S12" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1238,6 +1275,9 @@
       <c r="R14" t="n">
         <v>-175500</v>
       </c>
+      <c r="S14" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1299,6 +1339,9 @@
       </c>
       <c r="R15" t="n">
         <v>229860</v>
+      </c>
+      <c r="S15" t="n">
+        <v>1415</v>
       </c>
     </row>
     <row r="16">
@@ -1356,6 +1399,9 @@
       <c r="R16" t="n">
         <v>-232550</v>
       </c>
+      <c r="S16" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1418,6 +1464,9 @@
       <c r="R17" t="n">
         <v>60000</v>
       </c>
+      <c r="S17" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1479,6 +1528,9 @@
       </c>
       <c r="R18" t="n">
         <v>-2451</v>
+      </c>
+      <c r="S18" t="n">
+        <v>1415</v>
       </c>
     </row>
     <row r="19">
@@ -1532,6 +1584,9 @@
       <c r="R19" t="n">
         <v>344105</v>
       </c>
+      <c r="S19" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1594,6 +1649,9 @@
       <c r="R20" t="n">
         <v>72080</v>
       </c>
+      <c r="S20" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1656,6 +1714,7 @@
       <c r="R21" s="2" t="n">
         <v>295544</v>
       </c>
+      <c r="S21" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1696,6 +1755,7 @@
       <c r="R23" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S23" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1736,6 +1796,7 @@
       <c r="R25" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S25" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1776,6 +1837,7 @@
       <c r="R27" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S27" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1837,6 +1899,9 @@
       </c>
       <c r="R29" t="n">
         <v>-4553</v>
+      </c>
+      <c r="S29" t="n">
+        <v>1415</v>
       </c>
     </row>
     <row r="30">
@@ -1890,6 +1955,9 @@
       <c r="R30" t="n">
         <v>115600</v>
       </c>
+      <c r="S30" t="n">
+        <v>1411</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1952,6 +2020,7 @@
       <c r="R31" s="2" t="n">
         <v>111047</v>
       </c>
+      <c r="S31" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2008,6 +2077,9 @@
       <c r="R33" t="n">
         <v>-15508</v>
       </c>
+      <c r="S33" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2069,6 +2141,9 @@
       </c>
       <c r="R34" t="n">
         <v>-47176</v>
+      </c>
+      <c r="S34" t="n">
+        <v>1415</v>
       </c>
     </row>
     <row r="35">
@@ -2126,6 +2201,9 @@
       <c r="R35" t="n">
         <v>-1854</v>
       </c>
+      <c r="S35" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2178,6 +2256,9 @@
       <c r="R36" t="n">
         <v>52794</v>
       </c>
+      <c r="S36" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2220,19 +2301,22 @@
         <v>-0.864</v>
       </c>
       <c r="N37" t="n">
-        <v>-29079</v>
+        <v>-28997</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
       </c>
       <c r="P37" t="n">
-        <v>-87237</v>
+        <v>-86990</v>
       </c>
       <c r="Q37" t="n">
-        <v>13827</v>
+        <v>13787</v>
       </c>
       <c r="R37" t="n">
-        <v>-73410</v>
+        <v>-73203</v>
+      </c>
+      <c r="S37" t="n">
+        <v>1411</v>
       </c>
     </row>
     <row r="38">
@@ -2282,20 +2366,21 @@
         <v>-0.416</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-8042</v>
+        <v>-8024</v>
       </c>
       <c r="O38" s="2" t="n">
         <v>0.31</v>
       </c>
       <c r="P38" s="2" t="n">
-        <v>-112585</v>
+        <v>-112338</v>
       </c>
       <c r="Q38" s="2" t="n">
-        <v>27430</v>
+        <v>27391</v>
       </c>
       <c r="R38" s="2" t="n">
-        <v>-85155</v>
-      </c>
+        <v>-84947</v>
+      </c>
+      <c r="S38" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2358,6 +2443,9 @@
       <c r="R40" t="n">
         <v>15210</v>
       </c>
+      <c r="S40" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2420,6 +2508,9 @@
       <c r="R41" t="n">
         <v>-54359</v>
       </c>
+      <c r="S41" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2482,6 +2573,9 @@
       <c r="R42" t="n">
         <v>40095</v>
       </c>
+      <c r="S42" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2544,6 +2638,9 @@
       <c r="R43" t="n">
         <v>52844</v>
       </c>
+      <c r="S43" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2606,6 +2703,9 @@
       <c r="R44" t="n">
         <v>46340</v>
       </c>
+      <c r="S44" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2668,6 +2768,9 @@
       <c r="R45" t="n">
         <v>15177</v>
       </c>
+      <c r="S45" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2730,6 +2833,7 @@
       <c r="R46" s="2" t="n">
         <v>115307</v>
       </c>
+      <c r="S46" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2786,6 +2890,9 @@
       <c r="R48" t="n">
         <v>-13350</v>
       </c>
+      <c r="S48" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2842,6 +2949,7 @@
       <c r="R49" s="2" t="n">
         <v>-13350</v>
       </c>
+      <c r="S49" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2898,6 +3006,9 @@
       <c r="R51" t="n">
         <v>-133875</v>
       </c>
+      <c r="S51" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2954,6 +3065,7 @@
       <c r="R52" s="2" t="n">
         <v>-133875</v>
       </c>
+      <c r="S52" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3016,6 +3128,9 @@
       <c r="R54" t="n">
         <v>-77775</v>
       </c>
+      <c r="S54" t="n">
+        <v>1415</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3078,11 +3193,12 @@
       <c r="R55" s="2" t="n">
         <v>-77775</v>
       </c>
+      <c r="S55" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>5minHL</t>
+          <t>삼닉v3_미분류</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -3118,11 +3234,12 @@
       <c r="R57" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S57" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>5minHL2</t>
+          <t>5minHL</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -3158,11 +3275,12 @@
       <c r="R59" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S59" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>5minHL_동시</t>
+          <t>5minHL2</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -3198,124 +3316,48 @@
       <c r="R61" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S61" s="2" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>5minHL_미분류</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>5minHL_동시</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>분</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>06/22~06/26</t>
-        </is>
-      </c>
-      <c r="D63" t="n">
-        <v>1</v>
-      </c>
-      <c r="E63" t="n">
-        <v>0</v>
-      </c>
-      <c r="F63" t="n">
-        <v>0</v>
-      </c>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="n">
-        <v>49.85</v>
-      </c>
-      <c r="M63" t="n">
-        <v>-2.747</v>
-      </c>
-      <c r="N63" t="n">
-        <v>-2426</v>
-      </c>
-      <c r="O63" t="n">
-        <v>0</v>
-      </c>
-      <c r="P63" t="n">
-        <v>-2426</v>
-      </c>
-      <c r="Q63" t="n">
-        <v>26</v>
-      </c>
-      <c r="R63" t="n">
-        <v>-2400</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>5minHL_미분류</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>분</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>06/29~07/03</t>
-        </is>
-      </c>
-      <c r="D64" t="n">
-        <v>6</v>
-      </c>
-      <c r="E64" t="n">
-        <v>50</v>
-      </c>
-      <c r="F64" t="n">
-        <v>2.93</v>
-      </c>
-      <c r="G64" t="n">
-        <v>2.47</v>
-      </c>
-      <c r="H64" t="n">
-        <v>2.85</v>
-      </c>
-      <c r="I64" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="J64" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="K64" t="n">
-        <v>1279.97</v>
-      </c>
-      <c r="L64" t="n">
-        <v>875.09</v>
-      </c>
-      <c r="M64" t="n">
-        <v>-0.191</v>
-      </c>
-      <c r="N64" t="n">
-        <v>4951</v>
-      </c>
-      <c r="O64" t="n">
-        <v>2.93</v>
-      </c>
-      <c r="P64" t="n">
-        <v>29704</v>
-      </c>
-      <c r="Q64" t="n">
-        <v>756</v>
-      </c>
-      <c r="R64" t="n">
-        <v>30460</v>
-      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" s="2" t="inlineStr"/>
+      <c r="F63" s="2" t="inlineStr"/>
+      <c r="G63" s="2" t="inlineStr"/>
+      <c r="H63" s="2" t="inlineStr"/>
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr"/>
+      <c r="L63" s="2" t="inlineStr"/>
+      <c r="M63" s="2" t="inlineStr"/>
+      <c r="N63" s="2" t="inlineStr"/>
+      <c r="O63" s="2" t="inlineStr"/>
+      <c r="P63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S63" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3330,53 +3372,50 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>07/06~07/10</t>
+          <t>06/22~06/26</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E65" t="n">
-        <v>33.3</v>
+        <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G65" t="n">
-        <v>0.08</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G65" t="inlineStr"/>
       <c r="H65" t="n">
-        <v>3.13</v>
-      </c>
-      <c r="I65" t="n">
-        <v>0.08</v>
-      </c>
+        <v>2.75</v>
+      </c>
+      <c r="I65" t="inlineStr"/>
       <c r="J65" t="n">
-        <v>3.61</v>
-      </c>
-      <c r="K65" t="n">
-        <v>4319.93</v>
-      </c>
+        <v>2.75</v>
+      </c>
+      <c r="K65" t="inlineStr"/>
       <c r="L65" t="n">
-        <v>1351.81</v>
+        <v>49.85</v>
       </c>
       <c r="M65" t="n">
-        <v>-2.059</v>
+        <v>-2.747</v>
       </c>
       <c r="N65" t="n">
-        <v>-3794</v>
+        <v>-2426</v>
       </c>
       <c r="O65" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="P65" t="n">
-        <v>-11383</v>
+        <v>-2426</v>
       </c>
       <c r="Q65" t="n">
-        <v>153</v>
+        <v>26</v>
       </c>
       <c r="R65" t="n">
-        <v>-11230</v>
+        <v>-2400</v>
+      </c>
+      <c r="S65" t="n">
+        <v>1415</v>
       </c>
     </row>
     <row r="66">
@@ -3392,43 +3431,56 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>07/20~07/24</t>
+          <t>06/29~07/03</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E66" t="n">
-        <v>100</v>
-      </c>
-      <c r="F66" t="inlineStr"/>
+        <v>50</v>
+      </c>
+      <c r="F66" t="n">
+        <v>2.93</v>
+      </c>
       <c r="G66" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="H66" t="inlineStr"/>
+        <v>2.47</v>
+      </c>
+      <c r="H66" t="n">
+        <v>2.85</v>
+      </c>
       <c r="I66" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="J66" t="inlineStr"/>
+        <v>4.6</v>
+      </c>
+      <c r="J66" t="n">
+        <v>3.5</v>
+      </c>
       <c r="K66" t="n">
-        <v>10.1</v>
-      </c>
-      <c r="L66" t="inlineStr"/>
+        <v>1279.97</v>
+      </c>
+      <c r="L66" t="n">
+        <v>875.09</v>
+      </c>
       <c r="M66" t="n">
-        <v>1.678</v>
+        <v>-0.191</v>
       </c>
       <c r="N66" t="n">
-        <v>1670</v>
-      </c>
-      <c r="O66" t="inlineStr"/>
+        <v>4951</v>
+      </c>
+      <c r="O66" t="n">
+        <v>2.93</v>
+      </c>
       <c r="P66" t="n">
-        <v>1670</v>
+        <v>29704</v>
       </c>
       <c r="Q66" t="n">
-        <v>30</v>
+        <v>756</v>
       </c>
       <c r="R66" t="n">
-        <v>1700</v>
+        <v>30460</v>
+      </c>
+      <c r="S66" t="n">
+        <v>1415</v>
       </c>
     </row>
     <row r="67">
@@ -3444,120 +3496,181 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
+          <t>07/06~07/10</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E67" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H67" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="J67" t="n">
+        <v>3.61</v>
+      </c>
+      <c r="K67" t="n">
+        <v>4319.93</v>
+      </c>
+      <c r="L67" t="n">
+        <v>1351.81</v>
+      </c>
+      <c r="M67" t="n">
+        <v>-2.059</v>
+      </c>
+      <c r="N67" t="n">
+        <v>-3794</v>
+      </c>
+      <c r="O67" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="P67" t="n">
+        <v>-11383</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>153</v>
+      </c>
+      <c r="R67" t="n">
+        <v>-11230</v>
+      </c>
+      <c r="S67" t="n">
+        <v>1415</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>5minHL_미분류</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>분</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>07/20~07/24</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" t="n">
+        <v>100</v>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="n">
+        <v>1.678</v>
+      </c>
+      <c r="N68" t="n">
+        <v>1670</v>
+      </c>
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="n">
+        <v>1670</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>30</v>
+      </c>
+      <c r="R68" t="n">
+        <v>1700</v>
+      </c>
+      <c r="S68" t="n">
+        <v>1415</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>5minHL_미분류</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>분</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
           <t>07/27~07/31</t>
         </is>
       </c>
-      <c r="D67" t="n">
+      <c r="D69" t="n">
         <v>2</v>
       </c>
-      <c r="E67" t="n">
-        <v>0</v>
-      </c>
-      <c r="F67" t="n">
-        <v>0</v>
-      </c>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="n">
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="n">
         <v>6.78</v>
       </c>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="n">
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="n">
         <v>7.52</v>
       </c>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="n">
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="n">
         <v>5756.96</v>
       </c>
-      <c r="M67" t="n">
+      <c r="M69" t="n">
         <v>-6.785</v>
       </c>
-      <c r="N67" t="n">
+      <c r="N69" t="n">
         <v>-7272</v>
       </c>
-      <c r="O67" t="n">
-        <v>0</v>
-      </c>
-      <c r="P67" t="n">
+      <c r="O69" t="n">
+        <v>0</v>
+      </c>
+      <c r="P69" t="n">
         <v>-14543</v>
       </c>
-      <c r="Q67" t="n">
+      <c r="Q69" t="n">
         <v>58</v>
       </c>
-      <c r="R67" t="n">
+      <c r="R69" t="n">
         <v>-14485</v>
       </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>5minHL_미분류</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>분</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>전체</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="E68" s="2" t="n">
-        <v>38.5</v>
-      </c>
-      <c r="F68" s="2" t="n">
-        <v>1.71</v>
-      </c>
-      <c r="G68" s="2" t="n">
-        <v>1.83</v>
-      </c>
-      <c r="H68" s="2" t="n">
-        <v>3.89</v>
-      </c>
-      <c r="I68" s="2" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="J68" s="2" t="n">
-        <v>7.52</v>
-      </c>
-      <c r="K68" s="2" t="n">
-        <v>1633.99</v>
-      </c>
-      <c r="L68" s="2" t="n">
-        <v>2111.58</v>
-      </c>
-      <c r="M68" s="2" t="n">
-        <v>-1.689</v>
-      </c>
-      <c r="N68" s="2" t="n">
-        <v>232</v>
-      </c>
-      <c r="O68" s="2" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="P68" s="2" t="n">
-        <v>3022</v>
-      </c>
-      <c r="Q68" s="2" t="n">
-        <v>1023</v>
-      </c>
-      <c r="R68" s="2" t="n">
-        <v>4045</v>
+      <c r="S69" t="n">
+        <v>1415</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>KR_TR_ORD_A</t>
+          <t>5minHL_미분류</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>일</t>
+          <t>분</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -3566,33 +3679,56 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E70" s="2" t="inlineStr"/>
-      <c r="F70" s="2" t="inlineStr"/>
-      <c r="G70" s="2" t="inlineStr"/>
-      <c r="H70" s="2" t="inlineStr"/>
-      <c r="I70" s="2" t="inlineStr"/>
-      <c r="J70" s="2" t="inlineStr"/>
-      <c r="K70" s="2" t="inlineStr"/>
-      <c r="L70" s="2" t="inlineStr"/>
-      <c r="M70" s="2" t="inlineStr"/>
-      <c r="N70" s="2" t="inlineStr"/>
-      <c r="O70" s="2" t="inlineStr"/>
+        <v>13</v>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="H70" s="2" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="I70" s="2" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="J70" s="2" t="n">
+        <v>7.52</v>
+      </c>
+      <c r="K70" s="2" t="n">
+        <v>1633.99</v>
+      </c>
+      <c r="L70" s="2" t="n">
+        <v>2111.58</v>
+      </c>
+      <c r="M70" s="2" t="n">
+        <v>-1.689</v>
+      </c>
+      <c r="N70" s="2" t="n">
+        <v>232</v>
+      </c>
+      <c r="O70" s="2" t="n">
+        <v>1.07</v>
+      </c>
       <c r="P70" s="2" t="n">
-        <v>0</v>
+        <v>3022</v>
       </c>
       <c r="Q70" s="2" t="n">
-        <v>0</v>
+        <v>1023</v>
       </c>
       <c r="R70" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>4045</v>
+      </c>
+      <c r="S70" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>KR_TR_VOLUME_1</t>
+          <t>KR_TR_ORD_A</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3628,11 +3764,12 @@
       <c r="R72" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S72" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>KR_TR_VOLUME_2</t>
+          <t>KR_TR_VOLUME_1</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -3668,11 +3805,12 @@
       <c r="R74" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S74" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>KR_TR_VCP1</t>
+          <t>KR_TR_VOLUME_2</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -3708,11 +3846,12 @@
       <c r="R76" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S76" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>KR_TR_VCP2</t>
+          <t>KR_TR_VCP1</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -3748,11 +3887,12 @@
       <c r="R78" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S78" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>KR_TR_JEO2</t>
+          <t>KR_TR_VCP2</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -3788,11 +3928,12 @@
       <c r="R80" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S80" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>KR_TR_MA</t>
+          <t>KR_TR_JEO2</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -3828,11 +3969,12 @@
       <c r="R82" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S82" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>미국VCP</t>
+          <t>KR_TR_MA</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -3868,163 +4010,153 @@
       <c r="R84" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S84" s="2" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>KR_TR_ADD1</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr"/>
+      <c r="G86" s="2" t="inlineStr"/>
+      <c r="H86" s="2" t="inlineStr"/>
+      <c r="I86" s="2" t="inlineStr"/>
+      <c r="J86" s="2" t="inlineStr"/>
+      <c r="K86" s="2" t="inlineStr"/>
+      <c r="L86" s="2" t="inlineStr"/>
+      <c r="M86" s="2" t="inlineStr"/>
+      <c r="N86" s="2" t="inlineStr"/>
+      <c r="O86" s="2" t="inlineStr"/>
+      <c r="P86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S86" s="2" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>미국VCP</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr"/>
+      <c r="G88" s="2" t="inlineStr"/>
+      <c r="H88" s="2" t="inlineStr"/>
+      <c r="I88" s="2" t="inlineStr"/>
+      <c r="J88" s="2" t="inlineStr"/>
+      <c r="K88" s="2" t="inlineStr"/>
+      <c r="L88" s="2" t="inlineStr"/>
+      <c r="M88" s="2" t="inlineStr"/>
+      <c r="N88" s="2" t="inlineStr"/>
+      <c r="O88" s="2" t="inlineStr"/>
+      <c r="P88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S88" s="2" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
         <is>
           <t>US_TR_ORD_A</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B90" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C90" t="inlineStr">
         <is>
           <t>08/10~08/14</t>
         </is>
       </c>
-      <c r="D86" t="n">
+      <c r="D90" t="n">
         <v>1</v>
       </c>
-      <c r="E86" t="n">
-        <v>0</v>
-      </c>
-      <c r="F86" t="n">
-        <v>0</v>
-      </c>
-      <c r="G86" t="inlineStr"/>
-      <c r="H86" t="n">
+      <c r="E90" t="n">
+        <v>0</v>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="n">
         <v>10.01</v>
       </c>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="n">
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="n">
         <v>10.01</v>
       </c>
-      <c r="K86" t="inlineStr"/>
-      <c r="L86" t="n">
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="n">
         <v>3</v>
       </c>
-      <c r="M86" t="n">
+      <c r="M90" t="n">
         <v>-10.012</v>
       </c>
-      <c r="N86" t="n">
-        <v>-71616</v>
-      </c>
-      <c r="O86" t="n">
-        <v>0</v>
-      </c>
-      <c r="P86" t="n">
-        <v>-71616</v>
-      </c>
-      <c r="Q86" t="n">
-        <v>951</v>
-      </c>
-      <c r="R86" t="n">
-        <v>-70665</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="2" t="inlineStr">
-        <is>
-          <t>US_TR_ORD_A</t>
-        </is>
-      </c>
-      <c r="B87" s="2" t="inlineStr">
-        <is>
-          <t>일</t>
-        </is>
-      </c>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t>전체</t>
-        </is>
-      </c>
-      <c r="D87" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E87" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F87" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G87" s="2" t="inlineStr"/>
-      <c r="H87" s="2" t="n">
-        <v>10.01</v>
-      </c>
-      <c r="I87" s="2" t="inlineStr"/>
-      <c r="J87" s="2" t="n">
-        <v>10.01</v>
-      </c>
-      <c r="K87" s="2" t="inlineStr"/>
-      <c r="L87" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="M87" s="2" t="n">
-        <v>-10.012</v>
-      </c>
-      <c r="N87" s="2" t="n">
-        <v>-71616</v>
-      </c>
-      <c r="O87" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P87" s="2" t="n">
-        <v>-71616</v>
-      </c>
-      <c r="Q87" s="2" t="n">
-        <v>951</v>
-      </c>
-      <c r="R87" s="2" t="n">
-        <v>-70665</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="2" t="inlineStr">
-        <is>
-          <t>US_TR_VOLUME_1</t>
-        </is>
-      </c>
-      <c r="B89" s="2" t="inlineStr">
-        <is>
-          <t>일</t>
-        </is>
-      </c>
-      <c r="C89" s="2" t="inlineStr">
-        <is>
-          <t>전체</t>
-        </is>
-      </c>
-      <c r="D89" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E89" s="2" t="inlineStr"/>
-      <c r="F89" s="2" t="inlineStr"/>
-      <c r="G89" s="2" t="inlineStr"/>
-      <c r="H89" s="2" t="inlineStr"/>
-      <c r="I89" s="2" t="inlineStr"/>
-      <c r="J89" s="2" t="inlineStr"/>
-      <c r="K89" s="2" t="inlineStr"/>
-      <c r="L89" s="2" t="inlineStr"/>
-      <c r="M89" s="2" t="inlineStr"/>
-      <c r="N89" s="2" t="inlineStr"/>
-      <c r="O89" s="2" t="inlineStr"/>
-      <c r="P89" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q89" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R89" s="2" t="n">
-        <v>0</v>
+      <c r="N90" t="n">
+        <v>-71414</v>
+      </c>
+      <c r="O90" t="n">
+        <v>0</v>
+      </c>
+      <c r="P90" t="n">
+        <v>-71414</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>949</v>
+      </c>
+      <c r="R90" t="n">
+        <v>-70465</v>
+      </c>
+      <c r="S90" t="n">
+        <v>1411</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>US_TR_VOLUME_2</t>
+          <t>US_TR_ORD_A</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -4038,33 +4170,50 @@
         </is>
       </c>
       <c r="D91" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E91" s="2" t="inlineStr"/>
-      <c r="F91" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G91" s="2" t="inlineStr"/>
-      <c r="H91" s="2" t="inlineStr"/>
+      <c r="H91" s="2" t="n">
+        <v>10.01</v>
+      </c>
       <c r="I91" s="2" t="inlineStr"/>
-      <c r="J91" s="2" t="inlineStr"/>
+      <c r="J91" s="2" t="n">
+        <v>10.01</v>
+      </c>
       <c r="K91" s="2" t="inlineStr"/>
-      <c r="L91" s="2" t="inlineStr"/>
-      <c r="M91" s="2" t="inlineStr"/>
-      <c r="N91" s="2" t="inlineStr"/>
-      <c r="O91" s="2" t="inlineStr"/>
+      <c r="L91" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M91" s="2" t="n">
+        <v>-10.012</v>
+      </c>
+      <c r="N91" s="2" t="n">
+        <v>-71414</v>
+      </c>
+      <c r="O91" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="P91" s="2" t="n">
-        <v>0</v>
+        <v>-71414</v>
       </c>
       <c r="Q91" s="2" t="n">
-        <v>0</v>
+        <v>949</v>
       </c>
       <c r="R91" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>-70465</v>
+      </c>
+      <c r="S91" s="2" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>US_TR_VCP1</t>
+          <t>US_TR_VOLUME_1</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -4100,163 +4249,153 @@
       <c r="R93" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S93" s="2" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>US_TR_VOLUME_2</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" s="2" t="inlineStr"/>
+      <c r="F95" s="2" t="inlineStr"/>
+      <c r="G95" s="2" t="inlineStr"/>
+      <c r="H95" s="2" t="inlineStr"/>
+      <c r="I95" s="2" t="inlineStr"/>
+      <c r="J95" s="2" t="inlineStr"/>
+      <c r="K95" s="2" t="inlineStr"/>
+      <c r="L95" s="2" t="inlineStr"/>
+      <c r="M95" s="2" t="inlineStr"/>
+      <c r="N95" s="2" t="inlineStr"/>
+      <c r="O95" s="2" t="inlineStr"/>
+      <c r="P95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S95" s="2" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>US_TR_VCP1</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" s="2" t="inlineStr"/>
+      <c r="F97" s="2" t="inlineStr"/>
+      <c r="G97" s="2" t="inlineStr"/>
+      <c r="H97" s="2" t="inlineStr"/>
+      <c r="I97" s="2" t="inlineStr"/>
+      <c r="J97" s="2" t="inlineStr"/>
+      <c r="K97" s="2" t="inlineStr"/>
+      <c r="L97" s="2" t="inlineStr"/>
+      <c r="M97" s="2" t="inlineStr"/>
+      <c r="N97" s="2" t="inlineStr"/>
+      <c r="O97" s="2" t="inlineStr"/>
+      <c r="P97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S97" s="2" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
         <is>
           <t>US_TR_VCP2</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="B99" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C99" t="inlineStr">
         <is>
           <t>08/10~08/14</t>
         </is>
       </c>
-      <c r="D95" t="n">
+      <c r="D99" t="n">
         <v>1</v>
       </c>
-      <c r="E95" t="n">
-        <v>0</v>
-      </c>
-      <c r="F95" t="n">
-        <v>0</v>
-      </c>
-      <c r="G95" t="inlineStr"/>
-      <c r="H95" t="n">
+      <c r="E99" t="n">
+        <v>0</v>
+      </c>
+      <c r="F99" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="n">
         <v>6.8</v>
       </c>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="n">
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="n">
         <v>6.8</v>
       </c>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="n">
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="n">
         <v>5</v>
       </c>
-      <c r="M95" t="n">
+      <c r="M99" t="n">
         <v>-6.802</v>
       </c>
-      <c r="N95" t="n">
-        <v>-9904</v>
-      </c>
-      <c r="O95" t="n">
-        <v>0</v>
-      </c>
-      <c r="P95" t="n">
-        <v>-9904</v>
-      </c>
-      <c r="Q95" t="n">
-        <v>197</v>
-      </c>
-      <c r="R95" t="n">
-        <v>-9707</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="2" t="inlineStr">
-        <is>
-          <t>US_TR_VCP2</t>
-        </is>
-      </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t>일</t>
-        </is>
-      </c>
-      <c r="C96" s="2" t="inlineStr">
-        <is>
-          <t>전체</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G96" s="2" t="inlineStr"/>
-      <c r="H96" s="2" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="I96" s="2" t="inlineStr"/>
-      <c r="J96" s="2" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="K96" s="2" t="inlineStr"/>
-      <c r="L96" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="M96" s="2" t="n">
-        <v>-6.802</v>
-      </c>
-      <c r="N96" s="2" t="n">
-        <v>-9904</v>
-      </c>
-      <c r="O96" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P96" s="2" t="n">
-        <v>-9904</v>
-      </c>
-      <c r="Q96" s="2" t="n">
-        <v>197</v>
-      </c>
-      <c r="R96" s="2" t="n">
-        <v>-9707</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="2" t="inlineStr">
-        <is>
-          <t>US_TR_JEO2</t>
-        </is>
-      </c>
-      <c r="B98" s="2" t="inlineStr">
-        <is>
-          <t>일</t>
-        </is>
-      </c>
-      <c r="C98" s="2" t="inlineStr">
-        <is>
-          <t>전체</t>
-        </is>
-      </c>
-      <c r="D98" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E98" s="2" t="inlineStr"/>
-      <c r="F98" s="2" t="inlineStr"/>
-      <c r="G98" s="2" t="inlineStr"/>
-      <c r="H98" s="2" t="inlineStr"/>
-      <c r="I98" s="2" t="inlineStr"/>
-      <c r="J98" s="2" t="inlineStr"/>
-      <c r="K98" s="2" t="inlineStr"/>
-      <c r="L98" s="2" t="inlineStr"/>
-      <c r="M98" s="2" t="inlineStr"/>
-      <c r="N98" s="2" t="inlineStr"/>
-      <c r="O98" s="2" t="inlineStr"/>
-      <c r="P98" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q98" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R98" s="2" t="n">
-        <v>0</v>
+      <c r="N99" t="n">
+        <v>-9876</v>
+      </c>
+      <c r="O99" t="n">
+        <v>0</v>
+      </c>
+      <c r="P99" t="n">
+        <v>-9876</v>
+      </c>
+      <c r="Q99" t="n">
+        <v>196</v>
+      </c>
+      <c r="R99" t="n">
+        <v>-9679</v>
+      </c>
+      <c r="S99" t="n">
+        <v>1411</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>US_TR_MA</t>
+          <t>US_TR_VCP2</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -4270,33 +4409,50 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E100" s="2" t="inlineStr"/>
-      <c r="F100" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F100" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="G100" s="2" t="inlineStr"/>
-      <c r="H100" s="2" t="inlineStr"/>
+      <c r="H100" s="2" t="n">
+        <v>6.8</v>
+      </c>
       <c r="I100" s="2" t="inlineStr"/>
-      <c r="J100" s="2" t="inlineStr"/>
+      <c r="J100" s="2" t="n">
+        <v>6.8</v>
+      </c>
       <c r="K100" s="2" t="inlineStr"/>
-      <c r="L100" s="2" t="inlineStr"/>
-      <c r="M100" s="2" t="inlineStr"/>
-      <c r="N100" s="2" t="inlineStr"/>
-      <c r="O100" s="2" t="inlineStr"/>
+      <c r="L100" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M100" s="2" t="n">
+        <v>-6.802</v>
+      </c>
+      <c r="N100" s="2" t="n">
+        <v>-9876</v>
+      </c>
+      <c r="O100" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="P100" s="2" t="n">
-        <v>0</v>
+        <v>-9876</v>
       </c>
       <c r="Q100" s="2" t="n">
-        <v>0</v>
+        <v>196</v>
       </c>
       <c r="R100" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>-9679</v>
+      </c>
+      <c r="S100" s="2" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>미국수동</t>
+          <t>US_TR_JEO2</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -4332,16 +4488,17 @@
       <c r="R102" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S102" s="2" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>저점사다리</t>
+          <t>US_TR_MA</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>분</t>
+          <t>일</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -4372,16 +4529,17 @@
       <c r="R104" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S104" s="2" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>기타(8042)</t>
+          <t>US_TR_ADD1</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>분</t>
+          <t>일</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -4412,6 +4570,253 @@
       <c r="R106" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="S106" s="2" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>US_TR_LEGACY</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E108" s="2" t="inlineStr"/>
+      <c r="F108" s="2" t="inlineStr"/>
+      <c r="G108" s="2" t="inlineStr"/>
+      <c r="H108" s="2" t="inlineStr"/>
+      <c r="I108" s="2" t="inlineStr"/>
+      <c r="J108" s="2" t="inlineStr"/>
+      <c r="K108" s="2" t="inlineStr"/>
+      <c r="L108" s="2" t="inlineStr"/>
+      <c r="M108" s="2" t="inlineStr"/>
+      <c r="N108" s="2" t="inlineStr"/>
+      <c r="O108" s="2" t="inlineStr"/>
+      <c r="P108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S108" s="2" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>US_TR_LEGACY_TREND</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E110" s="2" t="inlineStr"/>
+      <c r="F110" s="2" t="inlineStr"/>
+      <c r="G110" s="2" t="inlineStr"/>
+      <c r="H110" s="2" t="inlineStr"/>
+      <c r="I110" s="2" t="inlineStr"/>
+      <c r="J110" s="2" t="inlineStr"/>
+      <c r="K110" s="2" t="inlineStr"/>
+      <c r="L110" s="2" t="inlineStr"/>
+      <c r="M110" s="2" t="inlineStr"/>
+      <c r="N110" s="2" t="inlineStr"/>
+      <c r="O110" s="2" t="inlineStr"/>
+      <c r="P110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S110" s="2" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>US_TR_LEGACY_LOW</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E112" s="2" t="inlineStr"/>
+      <c r="F112" s="2" t="inlineStr"/>
+      <c r="G112" s="2" t="inlineStr"/>
+      <c r="H112" s="2" t="inlineStr"/>
+      <c r="I112" s="2" t="inlineStr"/>
+      <c r="J112" s="2" t="inlineStr"/>
+      <c r="K112" s="2" t="inlineStr"/>
+      <c r="L112" s="2" t="inlineStr"/>
+      <c r="M112" s="2" t="inlineStr"/>
+      <c r="N112" s="2" t="inlineStr"/>
+      <c r="O112" s="2" t="inlineStr"/>
+      <c r="P112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S112" s="2" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>미국수동</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E114" s="2" t="inlineStr"/>
+      <c r="F114" s="2" t="inlineStr"/>
+      <c r="G114" s="2" t="inlineStr"/>
+      <c r="H114" s="2" t="inlineStr"/>
+      <c r="I114" s="2" t="inlineStr"/>
+      <c r="J114" s="2" t="inlineStr"/>
+      <c r="K114" s="2" t="inlineStr"/>
+      <c r="L114" s="2" t="inlineStr"/>
+      <c r="M114" s="2" t="inlineStr"/>
+      <c r="N114" s="2" t="inlineStr"/>
+      <c r="O114" s="2" t="inlineStr"/>
+      <c r="P114" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q114" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R114" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S114" s="2" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>저점사다리</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>분</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E116" s="2" t="inlineStr"/>
+      <c r="F116" s="2" t="inlineStr"/>
+      <c r="G116" s="2" t="inlineStr"/>
+      <c r="H116" s="2" t="inlineStr"/>
+      <c r="I116" s="2" t="inlineStr"/>
+      <c r="J116" s="2" t="inlineStr"/>
+      <c r="K116" s="2" t="inlineStr"/>
+      <c r="L116" s="2" t="inlineStr"/>
+      <c r="M116" s="2" t="inlineStr"/>
+      <c r="N116" s="2" t="inlineStr"/>
+      <c r="O116" s="2" t="inlineStr"/>
+      <c r="P116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S116" s="2" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>기타(8042)</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>분</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E118" s="2" t="inlineStr"/>
+      <c r="F118" s="2" t="inlineStr"/>
+      <c r="G118" s="2" t="inlineStr"/>
+      <c r="H118" s="2" t="inlineStr"/>
+      <c r="I118" s="2" t="inlineStr"/>
+      <c r="J118" s="2" t="inlineStr"/>
+      <c r="K118" s="2" t="inlineStr"/>
+      <c r="L118" s="2" t="inlineStr"/>
+      <c r="M118" s="2" t="inlineStr"/>
+      <c r="N118" s="2" t="inlineStr"/>
+      <c r="O118" s="2" t="inlineStr"/>
+      <c r="P118" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q118" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R118" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S118" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>